<commit_message>
🎯 Strict Pure scan [2026-09-14]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -3266,7 +3266,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>399.84 - 409.23 DR DEMAND</t>
+          <t>399.83 - 409.23 DR DEMAND</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>10163.48 - 10582.66 DR DEMAND</t>
+          <t>10163.49 - 10582.66 DR DEMAND</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">

</xml_diff>

<commit_message>
🎯 Strict Pure scan [2026-10-02]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -2066,7 +2066,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>399.84 - 409.23 DR DEMAND</t>
+          <t>399.83 - 409.23 DR DEMAND</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1595.35 - 1664.74 RD SUPPLY</t>
+          <t>1595.35 - 1664.73 RD SUPPLY</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>803.32 - 821.11 DR DEMAND</t>
+          <t>803.34 - 821.13 DR DEMAND</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>101787.0 - 105025.92 DR DEMAND</t>
+          <t>101787.0 - 105025.94 DR DEMAND</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">

</xml_diff>

<commit_message>
🎯 Strict Pure scan [2026-10-05]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -2066,7 +2066,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>399.83 - 409.23 DR DEMAND</t>
+          <t>399.84 - 409.23 DR DEMAND</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1595.35 - 1664.73 RD SUPPLY</t>
+          <t>1595.35 - 1664.74 RD SUPPLY</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>101787.0 - 105025.94 DR DEMAND</t>
+          <t>101787.0 - 105025.93 DR DEMAND</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">

</xml_diff>

<commit_message>
🎯 Strict Pure scan [2026-10-12]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -3666,7 +3666,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2494.13 - 2528.7 DR DEMAND</t>
+          <t>2494.13 - 2528.69 DR DEMAND</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -5826,12 +5826,12 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>— NO ACTIVE ZONE —</t>
+          <t>855.18 - 875.51 DR DEMAND</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.0 C</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">

</xml_diff>

<commit_message>
🎯 Strict Pure scan [2026-10-20]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -1346,7 +1346,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>399.83 - 409.23 DR DEMAND</t>
+          <t>399.84 - 409.23 DR DEMAND</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2494.13 - 2528.7 DR DEMAND</t>
+          <t>2494.13 - 2528.69 DR DEMAND</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>10163.49 - 10582.66 DR DEMAND</t>
+          <t>10163.48 - 10582.66 DR DEMAND</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">

</xml_diff>